<commit_message>
Modified TPS26630 resistor values
</commit_message>
<xml_diff>
--- a/plc/docs/TPS2663x _TPS1663x_Design_Calculator_revB.xlsx
+++ b/plc/docs/TPS2663x _TPS1663x_Design_Calculator_revB.xlsx
@@ -9965,7 +9965,7 @@
         <v>125</v>
       </c>
       <c r="D66" s="26">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="E66" s="31" t="s">
         <v>101</v>
@@ -9981,7 +9981,7 @@
       </c>
       <c r="D67" s="17">
         <f>D66</f>
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="E67" s="28" t="s">
         <v>45</v>
@@ -10673,7 +10673,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="28" operator="equal" id="{00370033-007E-44D9-86A0-0009003A0059}">
+          <x14:cfRule type="cellIs" priority="28" operator="equal" id="{00970066-0025-4399-AEC1-001400D50041}">
             <xm:f>"YES"</xm:f>
             <x14:dxf>
               <fill>
@@ -10687,7 +10687,7 @@
           <xm:sqref>D56</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="29" operator="equal" id="{003100CD-003D-4F38-845A-0076005D001E}">
+          <x14:cfRule type="cellIs" priority="29" operator="equal" id="{00710058-00C2-4816-AF65-003500AA00FF}">
             <xm:f>"NO"</xm:f>
             <x14:dxf>
               <fill>
@@ -10701,7 +10701,7 @@
           <xm:sqref>D56</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="26" operator="lessThan" id="{009E005C-001E-4661-AA4A-00D80056001D}">
+          <x14:cfRule type="cellIs" priority="26" operator="lessThan" id="{00AD00A9-0097-4545-993C-0004006C00DD}">
             <xm:f>2</xm:f>
             <x14:dxf>
               <fill>
@@ -10715,7 +10715,7 @@
           <xm:sqref>D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="27" operator="greaterThan" id="{0013008B-006F-4BBA-A712-0033008B00B4}">
+          <x14:cfRule type="cellIs" priority="27" operator="greaterThan" id="{009900FF-001E-4E58-B89D-002D004700C4}">
             <xm:f>2</xm:f>
             <x14:dxf>
               <fill>
@@ -10729,7 +10729,7 @@
           <xm:sqref>D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="22" operator="lessThan" id="{003200BA-002C-4913-86E8-00F8009500A9}">
+          <x14:cfRule type="cellIs" priority="22" operator="lessThan" id="{00380024-001E-4839-9714-00B7001300F3}">
             <xm:f>4</xm:f>
             <x14:dxf>
               <fill>
@@ -10743,7 +10743,7 @@
           <xm:sqref>D75</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="23" operator="greaterThan" id="{008B00F2-00E4-436D-829B-001600300089}">
+          <x14:cfRule type="cellIs" priority="23" operator="greaterThan" id="{00F9004F-007E-4A1C-B425-0026005900C8}">
             <xm:f>4</xm:f>
             <x14:dxf>
               <fill>
@@ -10757,7 +10757,7 @@
           <xm:sqref>D75</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="14" operator="lessThan" id="{009D003A-0059-4DE9-B379-00FD00CB003A}">
+          <x14:cfRule type="cellIs" priority="14" operator="lessThan" id="{00AF00DC-000E-41EA-9B46-0065005300EA}">
             <xm:f>$D$34</xm:f>
             <x14:dxf>
               <fill>
@@ -10771,7 +10771,7 @@
           <xm:sqref>D47</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="15" operator="greaterThan" id="{008600B1-001B-4ADC-9843-008F006D00E4}">
+          <x14:cfRule type="cellIs" priority="15" operator="greaterThan" id="{001B0047-002A-4127-81FB-002B00090056}">
             <xm:f>$D$34</xm:f>
             <x14:dxf>
               <fill>
@@ -10785,7 +10785,7 @@
           <xm:sqref>D47</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="13" operator="greaterThan" id="{005F00F5-00C2-49D6-A722-000800AA00B0}">
+          <x14:cfRule type="cellIs" priority="13" operator="greaterThan" id="{00E400AF-00CB-421C-B7F4-00A700FE003E}">
             <xm:f>6</xm:f>
             <x14:dxf>
               <fill>
@@ -10799,7 +10799,7 @@
           <xm:sqref>D15</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThan" id="{002A00EB-0013-4BF0-B6EF-0021000C00F2}">
+          <x14:cfRule type="cellIs" priority="11" operator="lessThan" id="{003D003A-0011-4853-A7A4-00C200D50025}">
             <xm:f>300</xm:f>
             <x14:dxf>
               <fill>
@@ -10813,7 +10813,7 @@
           <xm:sqref>D20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="greaterThan" id="{00260064-0001-4A42-A526-00C600E800DE}">
+          <x14:cfRule type="cellIs" priority="12" operator="greaterThan" id="{000400FE-0049-43AE-BC1C-006C00A00065}">
             <xm:f>300</xm:f>
             <x14:dxf>
               <fill>
@@ -10827,7 +10827,7 @@
           <xm:sqref>D20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="5" operator="containsText" text="NO" id="{00BF00D1-0076-4B0F-B943-00C500F4006E}">
+          <x14:cfRule type="containsText" priority="5" operator="containsText" text="NO" id="{00920095-00F9-4E54-AF4D-00B200290052}">
             <xm:f>NOT(ISERROR(SEARCH("NO",D68)))</xm:f>
             <x14:dxf>
               <fill>
@@ -10841,7 +10841,7 @@
           <xm:sqref>D68</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="6" operator="containsText" text="YES" id="{008E0056-0078-469C-9B6A-008200D90020}">
+          <x14:cfRule type="containsText" priority="6" operator="containsText" text="YES" id="{002D00F9-00B8-4008-AF50-0009003C00F8}">
             <xm:f>NOT(ISERROR(SEARCH("YES",D68)))</xm:f>
             <x14:dxf>
               <fill>
@@ -10855,7 +10855,7 @@
           <xm:sqref>D68</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="3" operator="lessThan" id="{0069009E-00D9-498A-8746-00EE00770084}">
+          <x14:cfRule type="cellIs" priority="3" operator="lessThan" id="{0032001D-00A8-4ECD-B5AA-006E00BB008D}">
             <xm:f>2</xm:f>
             <x14:dxf>
               <fill>
@@ -10869,7 +10869,7 @@
           <xm:sqref>D63</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="4" operator="greaterThan" id="{00D4002A-0095-4C66-B779-0030006500C2}">
+          <x14:cfRule type="cellIs" priority="4" operator="greaterThan" id="{002500FB-0080-42D2-AFA2-008100890048}">
             <xm:f>2</xm:f>
             <x14:dxf>
               <fill>
@@ -10883,7 +10883,7 @@
           <xm:sqref>D63</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{00860057-00F0-4866-9D13-001F00EF0089}">
+          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{009F008F-0034-49A7-B421-009F00AE00A9}">
             <xm:f>"YES"</xm:f>
             <x14:dxf>
               <fill>
@@ -10897,7 +10897,7 @@
           <xm:sqref>D55</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{00D500F4-00D3-4751-94BC-007D00D900CA}">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{00DD00A5-00AD-4F50-826F-00B400980070}">
             <xm:f>"NO"</xm:f>
             <x14:dxf>
               <fill>
@@ -10914,7 +10914,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="23" disablePrompts="0" xWindow="920" yWindow="270">
-        <x14:dataValidation xr:uid="{007E003D-00E8-49BC-8BCC-004900E3004A}" type="decimal" allowBlank="0" error="Enter a value in the range from 4.3V to VIN (min)" errorStyle="stop" errorTitle="UVSet Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
+        <x14:dataValidation xr:uid="{00040067-00DA-4DBC-A497-00BD00130068}" type="decimal" allowBlank="0" error="Enter a value in the range from 4.3V to VIN (min)" errorStyle="stop" errorTitle="UVSet Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
           <x14:formula1>
             <xm:f>4.5</xm:f>
           </x14:formula1>
@@ -10923,7 +10923,7 @@
           </x14:formula2>
           <xm:sqref>D8</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{008C0087-00AD-4F03-B00E-0082006E004D}" type="decimal" allowBlank="0" error="Enter a value greater than VIN(max) and less than 60V" errorStyle="stop" errorTitle="OVSet Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
+        <x14:dataValidation xr:uid="{0012005B-00F7-4669-9BF1-00FB00E90064}" type="decimal" allowBlank="0" error="Enter a value greater than VIN(max) and less than 60V" errorStyle="stop" errorTitle="OVSet Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
           <x14:formula1>
             <xm:f>D6</xm:f>
           </x14:formula1>
@@ -10932,13 +10932,13 @@
           </x14:formula2>
           <xm:sqref>D9</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00610089-007B-4897-8445-002400A7009C}" type="custom" allowBlank="1" error="Enter a value greater than (Vinmax / Maximum Load Current)" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" prompt="RLstart = Vinmax / Load Current during Start-up.&#10;If there is no load during startup, set RLstart to 1000" promptTitle="Tool Help" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{009F00EC-009F-4F2E-B624-001000FA00A5}" type="custom" allowBlank="1" error="Enter a value greater than (Vinmax / Maximum Load Current)" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" prompt="RLstart = Vinmax / Load Current during Start-up.&#10;If there is no load during startup, set RLstart to 1000" promptTitle="Tool Help" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>D12&gt;=(D6/D13)</xm:f>
           </x14:formula1>
           <xm:sqref>D12</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{0023007B-00BC-45D9-B4C7-00C700060054}" type="decimal" allowBlank="1" error="Enter a value in the range from 1k to 511k" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00B50066-00BD-434D-AC89-001700A00038}" type="decimal" allowBlank="1" error="Enter a value in the range from 1k to 511k" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>1</xm:f>
           </x14:formula1>
@@ -10947,7 +10947,7 @@
           </x14:formula2>
           <xm:sqref>D74</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00FA00DA-0035-44AD-8046-00F700C5009F}" type="decimal" allowBlank="1" error="Enter a value in the range from VIN(min) to VIN(max)." errorStyle="stop" errorTitle="VIN(nom) out of range " imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
+        <x14:dataValidation xr:uid="{00620091-0052-4FFE-AAB1-00EB002300D0}" type="decimal" allowBlank="1" error="Enter a value in the range from VIN(min) to VIN(max)." errorStyle="stop" errorTitle="VIN(nom) out of range " imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
           <x14:formula1>
             <xm:f>D5</xm:f>
           </x14:formula1>
@@ -10956,7 +10956,7 @@
           </x14:formula2>
           <xm:sqref>D7</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00A60032-0034-4B09-B462-00AD005C00A3}" type="decimal" allowBlank="1" error="Enter a value greater than Imax+ IINRUSH_permissible and less than 6A." errorStyle="stop" errorTitle="ILIM Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{002800B7-00F4-4D83-A7BE-0098008C003B}" type="decimal" allowBlank="1" error="Enter a value greater than Imax+ IINRUSH_permissible and less than 6A." errorStyle="stop" errorTitle="ILIM Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>D13+D14</xm:f>
           </x14:formula1>
@@ -10965,13 +10965,13 @@
           </x14:formula2>
           <xm:sqref>D15</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{002500D4-0031-40D1-A64A-00A8005600DB}" type="custom" allowBlank="0" error="CdVdT capacitor is not required if start-up time is less than or equal to default" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
+        <x14:dataValidation xr:uid="{009E00BC-0061-4966-B160-007500C700EE}" type="custom" allowBlank="0" error="CdVdT capacitor is not required if start-up time is less than or equal to default" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
           <x14:formula1>
             <xm:f>D40&gt;D38</xm:f>
           </x14:formula1>
           <xm:sqref>D40</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00F70033-0047-4C58-BDD0-00CB009C0037}" type="decimal" allowBlank="1" error="Enter a value in the range from 0.1V to 4V" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00610003-008D-4990-9FCA-002700D30001}" type="decimal" allowBlank="1" error="Enter a value in the range from 0.1V to 4V" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>0.01</xm:f>
           </x14:formula1>
@@ -10980,7 +10980,7 @@
           </x14:formula2>
           <xm:sqref>D71</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{000300B3-002C-4460-84C7-0052002B000C}" type="decimal" allowBlank="1" error="Enter a value between 0.1 to 33000uF" errorStyle="stop" errorTitle="Cout Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{007C0010-007E-4641-BC7B-00ED00EE00B0}" type="decimal" allowBlank="1" error="Enter a value between 0.1 to 33000uF" errorStyle="stop" errorTitle="Cout Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>0.1</xm:f>
           </x14:formula1>
@@ -10989,7 +10989,7 @@
           </x14:formula2>
           <xm:sqref>D10</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00700038-00DB-4C94-9F6D-00A900600089}" type="decimal" allowBlank="1" error="Enter a value in the range from 5.36k to 120k" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{008B00B7-00D8-419D-A243-002100A9000B}" type="decimal" allowBlank="1" error="Enter a value in the range from 5.36k to 120k" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>3</xm:f>
           </x14:formula1>
@@ -10998,13 +10998,13 @@
           </x14:formula2>
           <xm:sqref>D33</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{004A0027-00B7-4712-BDDA-00E300E10031}" type="decimal" allowBlank="1" error="Enter a value greater than or equal to  0.022uF" errorStyle="stop" imeMode="noControl" operator="greaterThanOrEqual" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{008E00A4-0064-4D8D-92C4-00A8002C009F}" type="decimal" allowBlank="1" error="Enter a value greater than or equal to  0.022uF" errorStyle="stop" imeMode="noControl" operator="greaterThanOrEqual" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>0.022</xm:f>
           </x14:formula1>
           <xm:sqref>D44</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{004600A2-008E-4D3A-AF4E-005A00F30053}" type="decimal" allowBlank="1" error="Enter a value in the range from 1k to 249k" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00080029-00DF-4158-8089-00DC00CB0038}" type="decimal" allowBlank="1" error="Enter a value in the range from 1k to 249k" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>1</xm:f>
           </x14:formula1>
@@ -11013,7 +11013,7 @@
           </x14:formula2>
           <xm:sqref>D18 D22:D23</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00AA001C-00B2-4321-8249-00FF00F500B9}" type="decimal" allowBlank="1" error="Enter a value in the range from 5% to 30%" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00A0008B-00C7-4D95-9B3D-00B7001700CE}" type="decimal" allowBlank="1" error="Enter a value in the range from 5% to 30%" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>0.05</xm:f>
           </x14:formula1>
@@ -11022,7 +11022,7 @@
           </x14:formula2>
           <xm:sqref>F10</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00D10016-0075-4CA0-8B99-003D00C50012}" type="decimal" allowBlank="1" error="Enter a value in the range from 0.1% to 10%" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00230099-00E6-4F84-8BFA-002F00AC0070}" type="decimal" allowBlank="1" error="Enter a value in the range from 0.1% to 10%" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>0.001</xm:f>
           </x14:formula1>
@@ -11031,7 +11031,7 @@
           </x14:formula2>
           <xm:sqref>F74 F18 F22:F24 F33</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{000400B3-00FA-47B1-BE05-00D300F90056}" type="decimal" allowBlank="1" error="Enter a value in the range from 2% to 20%" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00DE002D-00CD-47A6-9DB2-002900410012}" type="decimal" allowBlank="1" error="Enter a value in the range from 2% to 20%" errorStyle="stop" errorTitle="Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>0.02</xm:f>
           </x14:formula1>
@@ -11040,7 +11040,7 @@
           </x14:formula2>
           <xm:sqref>F44</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{0054006D-0052-489B-9BCE-00B0000D00ED}" type="decimal" allowBlank="1" error="Enter a value in the range from 0.6A to 5.7A" errorStyle="stop" errorTitle="Imax Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00B600F8-00D0-47E8-BEF0-00A600090098}" type="decimal" allowBlank="1" error="Enter a value in the range from 0.6A to 5.7A" errorStyle="stop" errorTitle="Imax Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>0.6</xm:f>
           </x14:formula1>
@@ -11049,7 +11049,7 @@
           </x14:formula2>
           <xm:sqref>D13</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00300013-0089-4B1E-B9DA-006D006C0047}" type="decimal" allowBlank="1" error="Enter a value Less than Imax and greater than 0.01A" errorStyle="stop" errorTitle="INrush Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00E7001D-0051-4477-A933-00C500AF00E7}" type="decimal" allowBlank="1" error="Enter a value Less than Imax and greater than 0.01A" errorStyle="stop" errorTitle="INrush Error" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>0.01</xm:f>
           </x14:formula1>
@@ -11058,19 +11058,19 @@
           </x14:formula2>
           <xm:sqref>D14</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{001C00BF-00ED-44C6-94F1-00D70050004E}" type="decimal" allowBlank="1" error="Enter a value greater than 100k" errorStyle="stop" imeMode="noControl" operator="greaterThanOrEqual" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{004400A5-008E-4C32-99FD-00F5004C00FD}" type="decimal" allowBlank="1" error="Enter a value greater than 100k" errorStyle="stop" imeMode="noControl" operator="greaterThanOrEqual" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>100</xm:f>
           </x14:formula1>
           <xm:sqref>D60</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{007A009C-0038-498D-99D6-0085009200E7}" type="decimal" allowBlank="1" error="Enter a value less than VINnom x ILimit" errorStyle="stop" imeMode="noControl" operator="lessThanOrEqual" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00330053-0010-4B9B-B91B-00E300CE00CF}" type="decimal" allowBlank="1" error="Enter a value less than VINnom x ILimit" errorStyle="stop" imeMode="noControl" operator="lessThanOrEqual" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>D7*D13</xm:f>
           </x14:formula1>
           <xm:sqref>D113</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00E60036-000F-459F-8917-00A2004C0046}" type="decimal" allowBlank="1" error="Enter a value between 40k to 150k" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00B100B8-001C-4CCA-878C-002300FA0019}" type="decimal" allowBlank="1" error="Enter a value between 40k to 150k" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>40</xm:f>
           </x14:formula1>
@@ -11079,7 +11079,7 @@
           </x14:formula2>
           <xm:sqref>D66</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{007B00CB-0063-4B2D-B525-004F00A3007C}" type="decimal" allowBlank="1" error="Enter Value between 4.5 to 60V" errorStyle="stop" errorTitle="VIN(min) " imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00CC002A-004A-41CE-B9E5-002D007D00CB}" type="decimal" allowBlank="1" error="Enter Value between 4.5 to 60V" errorStyle="stop" errorTitle="VIN(min) " imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>4.5</xm:f>
           </x14:formula1>
@@ -11088,13 +11088,13 @@
           </x14:formula2>
           <xm:sqref>D5</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00760096-0029-478F-A2DB-006A00A200B3}" type="decimal" allowBlank="1" error="Enter a value greater than VIN(min)." errorStyle="stop" errorTitle="VIN(max)&gt;OVset" imeMode="noControl" operator="greaterThan" showDropDown="0" showErrorMessage="1" showInputMessage="0">
+        <x14:dataValidation xr:uid="{007C000C-00F3-4CAD-9624-004E001F0096}" type="decimal" allowBlank="1" error="Enter a value greater than VIN(min)." errorStyle="stop" errorTitle="VIN(max)&gt;OVset" imeMode="noControl" operator="greaterThan" showDropDown="0" showErrorMessage="1" showInputMessage="0">
           <x14:formula1>
             <xm:f>D5</xm:f>
           </x14:formula1>
           <xm:sqref>D6</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{009A00C3-00AB-4254-8338-000E001B00BC}" type="decimal" allowBlank="1" error="Enter a value less than VIN(min)" errorStyle="stop" errorTitle="PGSET Error" imeMode="noControl" operator="lessThan" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00180091-0045-40FF-963E-00F200EF00C2}" type="decimal" allowBlank="1" error="Enter a value less than VIN(min)" errorStyle="stop" errorTitle="PGSET Error" imeMode="noControl" operator="lessThan" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>D5</xm:f>
           </x14:formula1>

</xml_diff>